<commit_message>
Wizard: overall questions folded into each job (no quick check), over 3 hours with every job fitting becomes two Fast Fix visits, one request with a service request created for jobs that don't fit, summary splits fast-fixable from the rest
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0133CFkBs7tc5jvnd6GkpBqc
</commit_message>
<xml_diff>
--- a/fast-fix/top-100-home-jobs.xlsx
+++ b/fast-fix/top-100-home-jobs.xlsx
@@ -6933,7 +6933,7 @@
     <t xml:space="preserve">Knockout questions</t>
   </si>
   <si>
-    <t xml:space="preserve">The conditions in the last column are PLACEHOLDER copy for design. In the one-job-at-a-time (wizard) version each task shows its conditions as a short list and then ONE question, "Does all of this apply to your job?" (Yes means it fits Fast Fix). Column Q is the single question the other versions ask instead; the next column keeps the questions that were merged or dropped on the way. A No flags that one task: before booking, the member sees a page that separates the jobs that fit Fast Fix from the jobs that need a service request, and can book the fitting ones or send everything as one service request. The three overall questions (step ladder, swap or repair only with no gas/new wiring/moved water lines, have the part) are asked once for the whole visit and send the whole request to the team if they fail. Answers are not stored; they only route the request.</t>
+    <t xml:space="preserve">The conditions in the last column are PLACEHOLDER copy for design. In the one-job-at-a-time (wizard) version each task shows its conditions as a short list, then the same three overall conditions for every job (standard step ladder; only a swap or repair with no gas, new wiring or moved water lines; you have the part or fixture), then ONE question, "Does all of this apply to your job?" (Yes means it fits Fast Fix). There is no separate quick-check step in the wizard. Column Q is the single question the other versions ask instead; the next column keeps the questions that were merged or dropped on the way. A No flags that one task. Before booking, the member sees a page that separates the jobs that fit Fast Fix from the jobs that need a service request; everything goes in as one request, the fitting jobs are booked, and our team schedules the rest. When every job fits but the visit runs past 3 hours (up to 6), it is booked as two Fast Fix visits. Answers are not stored; they only route the request.</t>
   </si>
   <si>
     <t xml:space="preserve">Evidence limits (read this)</t>
@@ -8921,8 +8921,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="1" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="17" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Wizard: each vetting question on its own, titled sections (Eligible for Fast Fix / Requires Service Request), and a Service Request module on the confirmation page
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0133CFkBs7tc5jvnd6GkpBqc
</commit_message>
<xml_diff>
--- a/fast-fix/top-100-home-jobs.xlsx
+++ b/fast-fix/top-100-home-jobs.xlsx
@@ -87,7 +87,7 @@
     <t xml:space="preserve">Other candidate questions (not used in Fast Fix)</t>
   </si>
   <si>
-    <t xml:space="preserve">Conditions shown in the wizard (Fast Fix covers this job when...)</t>
+    <t xml:space="preserve">Questions shown in the wizard, each answered on its own (the 3 overall questions are added for every job)</t>
   </si>
   <si>
     <t xml:space="preserve">Hole or dent in the wall</t>
@@ -117,7 +117,7 @@
     <t xml:space="preserve">Is the hole smaller than about 6 inches across?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The hole is smaller than about 6 inches across</t>
+    <t xml:space="preserve">1. Is the hole smaller than about 6 inches across?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a ceiling fan</t>
@@ -147,8 +147,8 @@
     <t xml:space="preserve">Is there already a ceiling fan (not just a light) where the new fan goes?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There is already a ceiling fan (not just a light) where the new fan goes
-- The old fan is mounted solidly, with no wobble from the ceiling box</t>
+    <t xml:space="preserve">1. Is the old fan mounted solidly, with no wobble coming from the ceiling box?
+2. Is there already a ceiling fan (not just a light) where the new fan goes?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace an indoor ceiling or wall light</t>
@@ -175,8 +175,8 @@
     <t xml:space="preserve">Is there already a light fixture where the new one will go?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The new light is a simple ceiling or wall light, not a chandelier or fan
-- There is already a light fixture where the new one will go</t>
+    <t xml:space="preserve">1. Is the new light a simple ceiling or wall light, not a chandelier or fan?
+2. Is there already a light fixture where the new one will go?</t>
   </si>
   <si>
     <t xml:space="preserve">Running toilet</t>
@@ -203,7 +203,7 @@
     <t xml:space="preserve">Is the tank free of cracks, with no water leaking onto the floor?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The tank has no cracks and no water is leaking onto the floor</t>
+    <t xml:space="preserve">1. Is the tank free of cracks, with no water leaking onto the floor?</t>
   </si>
   <si>
     <t xml:space="preserve">Moldy or cracked tub, shower or sink caulk</t>
@@ -227,7 +227,7 @@
     <t xml:space="preserve">Is the wall around the tub or sink solid, with no soft spots or loose tiles?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The wall around the tub or sink is solid, with no soft spots or loose tiles</t>
+    <t xml:space="preserve">1. Is the wall around the tub or sink solid, with no soft spots or loose tiles?</t>
   </si>
   <si>
     <t xml:space="preserve">Install a smart thermostat</t>
@@ -251,8 +251,8 @@
     <t xml:space="preserve">Does the maker's compatibility checker say the new thermostat works with your system?</t>
   </si>
   <si>
-    <t xml:space="preserve">- Your system is central heating or AC, not electric baseboard heaters
-- The maker's compatibility checker says the new thermostat works with your system</t>
+    <t xml:space="preserve">1. Is your system central heating or AC, not electric baseboard heaters?
+2. Does the maker's compatibility checker say the new thermostat works with your system?</t>
   </si>
   <si>
     <t xml:space="preserve">Door sticks, rubs or won't latch</t>
@@ -279,7 +279,7 @@
     <t xml:space="preserve">Is the door itself in good shape, not warped or cracked?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The door itself is in good shape, not warped or cracked</t>
+    <t xml:space="preserve">1. Is the door itself in good shape, not warped or cracked?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a garbage disposal</t>
@@ -306,8 +306,8 @@
     <t xml:space="preserve">Is there already a disposal under this sink that you are replacing?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There is already a disposal under this sink that you are replacing
-- The new disposal is the same type as the old one, plug-in or hardwired</t>
+    <t xml:space="preserve">1. Is the new disposal the same type as the old one, plug-in or hardwired?
+2. Is there already a disposal under this sink that you are replacing?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a kitchen or bathroom faucet</t>
@@ -334,8 +334,8 @@
     <t xml:space="preserve">Does the new faucet use the same number of holes as your sink has now?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The shutoff valves under the sink turn and stop the water
-- The new faucet uses the same number of holes as your sink has now</t>
+    <t xml:space="preserve">1. Do the shutoff valves under the sink turn and stop the water?
+2. Does the new faucet use the same number of holes as your sink has now?</t>
   </si>
   <si>
     <t xml:space="preserve">Dripping or weak sink faucet</t>
@@ -359,7 +359,7 @@
     <t xml:space="preserve">Is the leak at the faucet spout or handle, not from the pipes below or the wall?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The leak is at the faucet spout or handle, not from the pipes below or the wall</t>
+    <t xml:space="preserve">1. Is the leak at the faucet spout or handle, not from the pipes below or the wall?</t>
   </si>
   <si>
     <t xml:space="preserve">Loose, cracked or worn outlet</t>
@@ -386,8 +386,8 @@
     <t xml:space="preserve">Is only this one outlet affected, with the breaker not tripping?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The outlet has no scorch marks, burning smell or heat
-- Only this one outlet is affected, and the breaker is not tripping</t>
+    <t xml:space="preserve">1. Is the outlet free of scorch marks, a burning smell or heat?
+2. Is only this one outlet affected, with the breaker not tripping?</t>
   </si>
   <si>
     <t xml:space="preserve">Scuffs and small paint touch-ups</t>
@@ -411,7 +411,7 @@
     <t xml:space="preserve">Is it a few patches or one small wall section, not a whole room?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The job is a few patches or one small wall section, not a whole room</t>
+    <t xml:space="preserve">1. Is it a few patches or one small wall section, not a whole room?</t>
   </si>
   <si>
     <t xml:space="preserve">Mount a TV on a drywall or wood wall</t>
@@ -442,9 +442,9 @@
 Is there already a power outlet near where the TV will hang?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The TV is 65 inches or smaller
-- The wall is regular drywall, not brick, stone or concrete
-- There is already a power outlet near where the TV will hang</t>
+    <t xml:space="preserve">1. Is the TV 65 inches or smaller?
+2. Is the wall regular drywall, not brick, stone or concrete?
+3. Is there already a power outlet near where the TV will hang?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a deadbolt or entry lock</t>
@@ -471,8 +471,8 @@
     <t xml:space="preserve">Is the new lock a standard key deadbolt or lockset, not a smart lock?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The new lock fits the existing holes in the door, with no new drilling
-- The new lock is a standard key deadbolt or lockset, not a smart lock</t>
+    <t xml:space="preserve">1. Does the new lock fit the existing holes in the door, with no new drilling?
+2. Is the new lock a standard key deadbolt or lockset, not a smart lock?</t>
   </si>
   <si>
     <t xml:space="preserve">Assemble other flat-pack furniture</t>
@@ -496,7 +496,7 @@
     <t xml:space="preserve">Is it one or two pieces, not a bed, desk, dresser or whole room set?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The job is one or two pieces, not a bed, desk, dresser or whole room set</t>
+    <t xml:space="preserve">1. Is it one or two pieces, not a bed, desk, dresser or whole room set?</t>
   </si>
   <si>
     <t xml:space="preserve">Hang shelves on the wall</t>
@@ -517,7 +517,7 @@
     <t xml:space="preserve">Is the wall plain drywall, not tile, brick or stone?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The wall is plain drywall, not tile, brick or stone</t>
+    <t xml:space="preserve">1. Is the wall plain drywall, not tile, brick or stone?</t>
   </si>
   <si>
     <t xml:space="preserve">Draft coming in around an outside door</t>
@@ -538,7 +538,7 @@
     <t xml:space="preserve">Is the gap just worn seals or a loose sweep, not a warped or damaged door?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The gap is from worn seals or a loose sweep, not a warped or damaged door</t>
+    <t xml:space="preserve">1. Is the gap just worn seals or a loose sweep, not a warped or damaged door?</t>
   </si>
   <si>
     <t xml:space="preserve">Clogged toilet</t>
@@ -565,8 +565,8 @@
     <t xml:space="preserve">Is this the first clog in a while, not a toilet that keeps clogging?</t>
   </si>
   <si>
-    <t xml:space="preserve">- Only this one toilet is backing up, and the sinks and tub drain fine
-- This is the first clog in a while, not a toilet that keeps clogging</t>
+    <t xml:space="preserve">1. Is only this one toilet backing up, with the sinks and tub draining fine?
+2. Is this the first clog in a while, not a toilet that keeps clogging?</t>
   </si>
   <si>
     <t xml:space="preserve">Broken light switch or add a dimmer</t>
@@ -590,7 +590,7 @@
     <t xml:space="preserve">Is there already a switch in this spot that you want swapped?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There is already a switch in this spot that you want swapped</t>
+    <t xml:space="preserve">1. Is there already a switch in this spot that you want swapped?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a toilet</t>
@@ -615,9 +615,9 @@
 Is the floor around the toilet firm, with no soft or spongy spots?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The water shutoff valve behind the toilet turns and stops the water
-- An adult helper is at home to help lift the old and new toilet
-- The floor around the toilet is firm, with no soft or spongy spots</t>
+    <t xml:space="preserve">1. Does the water shutoff valve behind the toilet turn and stop the water?
+2. Is there an adult helper at home to help lift the old and new toilet?
+3. Is the floor around the toilet firm, with no soft or spongy spots?</t>
   </si>
   <si>
     <t xml:space="preserve">Leak under the sink</t>
@@ -641,7 +641,7 @@
     <t xml:space="preserve">Is the drip at a pipe connection or hose under the sink, not inside the wall?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The drip is at a pipe connection or hose under the sink, not inside the wall</t>
+    <t xml:space="preserve">1. Is the drip at a pipe connection or hose under the sink, not inside the wall?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a broken or old door knob</t>
@@ -665,7 +665,7 @@
     <t xml:space="preserve">Is the new knob or lever a plain one that fits the existing hole in the door?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The new knob or lever is a plain one that fits the existing hole in the door</t>
+    <t xml:space="preserve">1. Is the new knob or lever a plain one that fits the existing hole in the door?</t>
   </si>
   <si>
     <t xml:space="preserve">Change the furnace or AC filter</t>
@@ -704,7 +704,7 @@
     <t xml:space="preserve">Is the new doorbell battery-powered, or is your current wired doorbell working?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The new doorbell is battery-powered, or your current wired doorbell works</t>
+    <t xml:space="preserve">1. Is the new doorbell battery-powered, or is your current wired doorbell working?</t>
   </si>
   <si>
     <t xml:space="preserve">Slow or clogged sink drain</t>
@@ -728,7 +728,7 @@
     <t xml:space="preserve">Is only this one sink slow, with the other drains in the house working fine?</t>
   </si>
   <si>
-    <t xml:space="preserve">- Only this one sink is slow, and the other drains in the house work fine</t>
+    <t xml:space="preserve">1. Is only this one sink slow, with the other drains in the house working fine?</t>
   </si>
   <si>
     <t xml:space="preserve">Hang pictures or wall art</t>
@@ -746,7 +746,7 @@
     <t xml:space="preserve">Is each frame or piece of art lighter than about 25 pounds?</t>
   </si>
   <si>
-    <t xml:space="preserve">- Each frame or piece of art is lighter than about 25 pounds</t>
+    <t xml:space="preserve">1. Is each frame or piece of art lighter than about 25 pounds?</t>
   </si>
   <si>
     <t xml:space="preserve">Install blinds or shades</t>
@@ -770,8 +770,8 @@
     <t xml:space="preserve">Are there six windows or fewer?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The blinds are ready-made stock sizes, not custom or motorized
-- There are six windows or fewer</t>
+    <t xml:space="preserve">1. Are the blinds ready-made stock sizes, not custom or motorized?
+2. Are there six windows or fewer?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a dishwasher</t>
@@ -796,9 +796,9 @@
 Can an adult helper be there to help lift the unit?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There is already a working shutoff valve under the sink
-- The new dishwasher is the same size and type as the old one
-- An adult helper can be there to help lift the unit</t>
+    <t xml:space="preserve">1. Is there already a working shutoff valve under the sink?
+2. Is the new dishwasher the same size and type as the old one?
+3. Can an adult helper be there to help lift the unit?</t>
   </si>
   <si>
     <t xml:space="preserve">Install a smart lock</t>
@@ -822,8 +822,8 @@
     <t xml:space="preserve">Does the current deadbolt slide into the frame smoothly?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There is already a standard deadbolt on the door with a drilled hole
-- The current deadbolt slides into the frame smoothly</t>
+    <t xml:space="preserve">1. Is there already a standard deadbolt on the door with a drilled hole?
+2. Does the current deadbolt slide into the frame smoothly?</t>
   </si>
   <si>
     <t xml:space="preserve">Change light bulbs too high to reach</t>
@@ -847,7 +847,7 @@
     <t xml:space="preserve">Is the fixture in a regular room, not a stairwell or two-story foyer?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The fixture is in a regular room, not a stairwell or two-story foyer</t>
+    <t xml:space="preserve">1. Is the fixture in a regular room, not a stairwell or two-story foyer?</t>
   </si>
   <si>
     <t xml:space="preserve">Slow or clogged shower or tub drain</t>
@@ -871,7 +871,7 @@
     <t xml:space="preserve">Are the other drains and toilets in the house working normally?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The other drains and toilets in the house are working normally</t>
+    <t xml:space="preserve">1. Are the other drains and toilets in the house working normally?</t>
   </si>
   <si>
     <t xml:space="preserve">Torn or damaged window screen</t>
@@ -892,7 +892,7 @@
     <t xml:space="preserve">Is the screen frame straight and sound, not badly bent or broken?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The screen frame is straight and sound, not badly bent or broken</t>
+    <t xml:space="preserve">1. Is the screen frame straight and sound, not badly bent or broken?</t>
   </si>
   <si>
     <t xml:space="preserve">Install wireless security cameras</t>
@@ -919,8 +919,8 @@
     <t xml:space="preserve">Are there three cameras or fewer?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The cameras are battery-powered or plug-in, with no wiring needed
-- There are three cameras or fewer</t>
+    <t xml:space="preserve">1. Are the cameras battery-powered or plug-in, with no wiring needed?
+2. Are there three cameras or fewer?</t>
   </si>
   <si>
     <t xml:space="preserve">Cold air leaking around a window</t>
@@ -944,8 +944,8 @@
     <t xml:space="preserve">Is the draft from worn seals or gaps, not a broken frame or glass?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The draft comes from worn seals or gaps, not a broken frame or glass
-- There are six windows or fewer</t>
+    <t xml:space="preserve">1. Is the draft from worn seals or gaps, not a broken frame or glass?
+2. Are there six windows or fewer?</t>
   </si>
   <si>
     <t xml:space="preserve">Dryer slow to dry or lint-clogged vent</t>
@@ -969,7 +969,7 @@
     <t xml:space="preserve">Does the dryer vent out of a nearby wall rather than through the attic or roof?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The dryer vents out of a nearby wall, not through the attic or roof</t>
+    <t xml:space="preserve">1. Does the dryer vent out of a nearby wall rather than through the attic or roof?</t>
   </si>
   <si>
     <t xml:space="preserve">Smoke or CO alarm is 10 years old</t>
@@ -996,8 +996,8 @@
     <t xml:space="preserve">Are there four alarms or fewer to replace?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The new alarms are the same type as the old ones (battery or plug-in)
-- There are four alarms or fewer to replace</t>
+    <t xml:space="preserve">1. Are the new alarms the same type as the old ones (battery or plug-in)?
+2. Are there four alarms or fewer to replace?</t>
   </si>
   <si>
     <t xml:space="preserve">Gaps around windows or doors</t>
@@ -1024,8 +1024,8 @@
     <t xml:space="preserve">Are there six windows or doors or fewer?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The wood around each opening is firm, not soft or rotted
-- There are six or fewer windows or doors</t>
+    <t xml:space="preserve">1. Is the wood around each opening firm, not soft or rotted?
+2. Are there six windows or doors or fewer?</t>
   </si>
   <si>
     <t xml:space="preserve">Hang curtain rods and curtains</t>
@@ -1046,8 +1046,8 @@
     <t xml:space="preserve">Are there three windows or fewer?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The rods are standard ready-made rods, not custom or motorized tracks
-- There are three windows or fewer</t>
+    <t xml:space="preserve">1. Are the rods standard ready-made rods, not custom or motorized tracks?
+2. Are there three windows or fewer?</t>
   </si>
   <si>
     <t xml:space="preserve">Outlet has no power or won't reset</t>
@@ -1074,8 +1074,8 @@
     <t xml:space="preserve">Has the breaker stayed on, without tripping again and again?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The outlet is cool to the touch, with no burning smell or scorch marks
-- The breaker has stayed on, without tripping again and again</t>
+    <t xml:space="preserve">1. Is the outlet cool to the touch, with no burning smell or scorch marks?
+2. Has the breaker stayed on, without tripping again and again?</t>
   </si>
   <si>
     <t xml:space="preserve">Sagging gate or broken fence boards</t>
@@ -1105,8 +1105,8 @@
     <t xml:space="preserve">Are only a few boards (about five or fewer) broken?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The gate post is solid, not leaning or loose in the ground
-- Only a few boards (about five or fewer) are broken</t>
+    <t xml:space="preserve">1. Is the gate post solid, not leaning or loose in the ground?
+2. Are only a few boards (about five or fewer) broken?</t>
   </si>
   <si>
     <t xml:space="preserve">Clogged or overflowing gutters</t>
@@ -1133,8 +1133,8 @@
     <t xml:space="preserve">Do you only need above-ground downspout extensions, with no digging?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The gutters are firmly attached, not sagging or pulling away
-- You only need above-ground downspout extensions, with no digging</t>
+    <t xml:space="preserve">1. Are the gutters firmly attached, not sagging or pulling away from the house?
+2. Do you only need above-ground downspout extensions, with no digging?</t>
   </si>
   <si>
     <t xml:space="preserve">Set up smart plugs or speakers</t>
@@ -1161,8 +1161,8 @@
     <t xml:space="preserve">Are there five devices or fewer to set up?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The devices are plug-in or battery types, with no hardwiring needed
-- There are five devices or fewer to set up</t>
+    <t xml:space="preserve">1. Are the devices plug-in or battery types, with no hardwiring needed?
+2. Are there five devices or fewer to set up?</t>
   </si>
   <si>
     <t xml:space="preserve">Window sticks or won't lock</t>
@@ -1183,7 +1183,7 @@
     <t xml:space="preserve">Are the glass and frame intact, with no cracks, rot or warping?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The glass and frame are intact, with no cracks, rot or warping</t>
+    <t xml:space="preserve">1. Are the glass and frame intact, with no cracks, rot or warping?</t>
   </si>
   <si>
     <t xml:space="preserve">Paint a door or accent wall</t>
@@ -1207,8 +1207,8 @@
     <t xml:space="preserve">Is the surface in good shape, with no peeling paint or holes to repair first?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The job is just one door or one wall, not a whole room
-- The surface is in good shape, with no peeling paint or holes to fix</t>
+    <t xml:space="preserve">1. Is the job just one door or one wall, not a whole room?
+2. Is the surface in good shape, with no peeling paint or holes to repair first?</t>
   </si>
   <si>
     <t xml:space="preserve">Bathroom fan noisy or not working</t>
@@ -1235,8 +1235,8 @@
     <t xml:space="preserve">Is the new fan the same size and type as the old one?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The old fan can be removed from below, with no attic access needed
-- The new fan is the same size and type as the old one</t>
+    <t xml:space="preserve">1. Can the old fan be removed from below, with no attic access needed?
+2. Is the new fan the same size and type as the old one?</t>
   </si>
   <si>
     <t xml:space="preserve">Cabinet door sags or drawer sticks</t>
@@ -1257,7 +1257,7 @@
     <t xml:space="preserve">Is the cabinet door or drawer itself intact, with no cracks or water damage?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The cabinet door or drawer itself is intact, with no cracks or water damage</t>
+    <t xml:space="preserve">1. Is the cabinet door or drawer itself intact, with no cracks or water damage?</t>
   </si>
   <si>
     <t xml:space="preserve">Mount a TV on a brick or stone wall</t>
@@ -1285,9 +1285,9 @@
 Is the TV going on a wall that is not above a fireplace?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The brick or stone is solid, not crumbling or a thin veneer
-- The TV is 65 inches or smaller
-- The TV is not going above a fireplace</t>
+    <t xml:space="preserve">1. Is the brick or stone solid, not crumbling or a thin veneer?
+2. Is the TV 65 inches or smaller?
+3. Is the TV going on a wall that is not above a fireplace?</t>
   </si>
   <si>
     <t xml:space="preserve">Install grab bars</t>
@@ -1311,8 +1311,8 @@
     <t xml:space="preserve">Are the bars rated to support a person's weight (not suction-cup bars)?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The wall is tile or drywall, not a thin fiberglass or acrylic shower surround
-- The bars are rated to support a person's weight, not suction-cup bars</t>
+    <t xml:space="preserve">1. Is the wall tile or drywall, not a thin fiberglass or acrylic shower surround?
+2. Are the bars rated to support a person's weight (not suction-cup bars)?</t>
   </si>
   <si>
     <t xml:space="preserve">Garage door won't close or remote fails</t>
@@ -1336,7 +1336,7 @@
     <t xml:space="preserve">Is the door itself working normally, with no broken spring or snapped cable?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The door itself works normally, with no broken spring or snapped cable</t>
+    <t xml:space="preserve">1. Is the door itself working normally, with no broken spring or snapped cable?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a showerhead</t>
@@ -1357,7 +1357,7 @@
     <t xml:space="preserve">Is the pipe arm that the showerhead screws onto solid, not loose or leaking?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The pipe arm the showerhead screws onto is solid, not loose or leaking</t>
+    <t xml:space="preserve">1. Is the pipe arm that the showerhead screws onto solid, not loose or leaking?</t>
   </si>
   <si>
     <t xml:space="preserve">Baby-proof cabinets and outlets</t>
@@ -1378,7 +1378,7 @@
     <t xml:space="preserve">Are there 15 or fewer cabinets and drawers to latch?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There are 15 or fewer cabinets and drawers to latch</t>
+    <t xml:space="preserve">1. Are there 15 or fewer cabinets and drawers to latch?</t>
   </si>
   <si>
     <t xml:space="preserve">Rotted or loose deck boards</t>
@@ -1405,8 +1405,8 @@
     <t xml:space="preserve">Are five or fewer deck boards damaged?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The deck is low to the ground with solid framing under the boards
-- Five or fewer deck boards are damaged</t>
+    <t xml:space="preserve">1. Is the deck low to the ground with solid framing under the boards?
+2. Are five or fewer deck boards damaged?</t>
   </si>
   <si>
     <t xml:space="preserve">Cracks or bumps in walls and ceilings</t>
@@ -1433,8 +1433,8 @@
     <t xml:space="preserve">Do nearby doors and windows still open and close normally?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The cracks are thin hairline cracks, not wide or stair-step
-- Nearby doors and windows still open and close normally</t>
+    <t xml:space="preserve">1. Are the cracks thin hairline cracks, not wide or stair-step?
+2. Do nearby doors and windows still open and close normally?</t>
   </si>
   <si>
     <t xml:space="preserve">Cracked or loose floor or wall tile</t>
@@ -1461,8 +1461,8 @@
     <t xml:space="preserve">Are three or fewer tiles cracked or loose?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The surface under the tile is firm and dry, not soft or damp
-- Three or fewer tiles are cracked or loose</t>
+    <t xml:space="preserve">1. Is the surface under the tile firm and dry, not soft or damp?
+2. Are three or fewer tiles cracked or loose?</t>
   </si>
   <si>
     <t xml:space="preserve">Garbage disposal jammed or humming</t>
@@ -1483,7 +1483,7 @@
     <t xml:space="preserve">Is the disposal jammed or humming, with no water leaking underneath?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The disposal is jammed or humming, with no water leaking underneath</t>
+    <t xml:space="preserve">1. Is the disposal jammed or humming, with no water leaking underneath?</t>
   </si>
   <si>
     <t xml:space="preserve">Change locks so old keys stop working</t>
@@ -1510,8 +1510,8 @@
     <t xml:space="preserve">Are there three or fewer locks to rekey?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The locks are standard knob or deadbolt locks, not smart or mortise locks
-- There are three or fewer locks to rekey</t>
+    <t xml:space="preserve">1. Are they standard knob or deadbolt locks, not smart or mortise locks?
+2. Are there three or fewer locks to rekey?</t>
   </si>
   <si>
     <t xml:space="preserve">Hang holiday lights or set up decor</t>
@@ -1538,8 +1538,8 @@
     <t xml:space="preserve">Is there an outdoor outlet near where the lights will go?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The lights are for the porch, bushes or low eaves, not the roofline
-- There is an outdoor outlet near where the lights will go</t>
+    <t xml:space="preserve">1. Are the lights for the porch, bushes or low eaves, not the roofline?
+2. Is there an outdoor outlet near where the lights will go?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace cabinet handles or hinges</t>
@@ -1563,8 +1563,8 @@
     <t xml:space="preserve">Are there 20 or fewer pieces of hardware to swap?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The new knobs or pulls fit the existing screw holes
-- There are 20 or fewer pieces of hardware to swap</t>
+    <t xml:space="preserve">1. Do the new knobs or pulls fit the existing screw holes?
+2. Are there 20 or fewer pieces of hardware to swap?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace an interior door</t>
@@ -1591,8 +1591,8 @@
     <t xml:space="preserve">Is the door frame square and undamaged, not rotted or warped?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The new door is the same size as the old one
-- The door frame is square and undamaged, not rotted or warped</t>
+    <t xml:space="preserve">1. Is the new door the same size as the old one?
+2. Is the door frame square and undamaged, not rotted or warped?</t>
   </si>
   <si>
     <t xml:space="preserve">Smoke or CO alarm chirping or beeping</t>
@@ -1616,7 +1616,7 @@
     <t xml:space="preserve">Are four or fewer alarms chirping?</t>
   </si>
   <si>
-    <t xml:space="preserve">- Four or fewer alarms are chirping</t>
+    <t xml:space="preserve">1. Are four or fewer alarms chirping?</t>
   </si>
   <si>
     <t xml:space="preserve">Outdoor faucet dripping or leaking</t>
@@ -1640,7 +1640,7 @@
     <t xml:space="preserve">Is the drip at the faucet handle or spout, not from the pipe in the wall?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The drip is at the faucet handle or spout, not from the pipe in the wall</t>
+    <t xml:space="preserve">1. Is the drip at the faucet handle or spout, not from the pipe in the wall?</t>
   </si>
   <si>
     <t xml:space="preserve">Dishwasher leaking or won't drain</t>
@@ -1664,7 +1664,7 @@
     <t xml:space="preserve">Is the dishwasher free of error codes and loud grinding noises?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The dishwasher has no error codes or loud grinding noises</t>
+    <t xml:space="preserve">1. Is the dishwasher free of error codes and loud grinding noises?</t>
   </si>
   <si>
     <t xml:space="preserve">Broken or cracked window glass</t>
@@ -1691,8 +1691,8 @@
     <t xml:space="preserve">Is the broken window on the ground floor?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is a single pane of glass, not a sealed double-pane unit
-- The broken window is on the ground floor</t>
+    <t xml:space="preserve">1. Is it a single pane of glass, not a sealed double-pane unit?
+2. Is the broken window on the ground floor?</t>
   </si>
   <si>
     <t xml:space="preserve">Install a closet rod or shelf</t>
@@ -1713,7 +1713,7 @@
     <t xml:space="preserve">Is it a single rod or shelf run in one closet or pantry?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is a single rod or shelf run in one closet or pantry</t>
+    <t xml:space="preserve">1. Is it a single rod or shelf run in one closet or pantry?</t>
   </si>
   <si>
     <t xml:space="preserve">Cracked or loose toilet seat</t>
@@ -1734,7 +1734,7 @@
     <t xml:space="preserve">Is it just the seat that is loose or broken, not the toilet itself?</t>
   </si>
   <si>
-    <t xml:space="preserve">- Only the seat is loose or broken, not the toilet itself</t>
+    <t xml:space="preserve">1. Is it just the seat that is loose or broken, not the toilet itself?</t>
   </si>
   <si>
     <t xml:space="preserve">Assemble a desk</t>
@@ -1752,7 +1752,7 @@
     <t xml:space="preserve">Is it one desk, not a multi-piece office suite?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is one desk, not a multi-piece office suite</t>
+    <t xml:space="preserve">1. Is it one desk, not a multi-piece office suite?</t>
   </si>
   <si>
     <t xml:space="preserve">Hang a heavy mirror</t>
@@ -1770,7 +1770,7 @@
     <t xml:space="preserve">Is the mirror 50 pounds or less?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The mirror weighs 50 pounds or less</t>
+    <t xml:space="preserve">1. Is the mirror 50 pounds or less?</t>
   </si>
   <si>
     <t xml:space="preserve">Mount and connect a soundbar</t>
@@ -1791,7 +1791,7 @@
     <t xml:space="preserve">Is it just a soundbar, with no in-wall wire or surround speakers?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is just a soundbar, with no in-wall wire or surround speakers</t>
+    <t xml:space="preserve">1. Is it just a soundbar, with no in-wall wire or surround speakers?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a microwave above the stove</t>
@@ -1818,8 +1818,8 @@
     <t xml:space="preserve">Is the new microwave the same width as the old one?</t>
   </si>
   <si>
-    <t xml:space="preserve">- A microwave is already mounted over the stove, with an outlet above it
-- The new microwave is the same width as the old one</t>
+    <t xml:space="preserve">1. Is a microwave already mounted over the stove, with an outlet above it?
+2. Is the new microwave the same width as the old one?</t>
   </si>
   <si>
     <t xml:space="preserve">Storm or screen door won't close or latch</t>
@@ -1843,8 +1843,7 @@
     <t xml:space="preserve">Is the door frame square and undamaged, with only the closer, latch or screen worn?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The door frame is square and undamaged
-- Only the closer, latch or screen is worn</t>
+    <t xml:space="preserve">1. Is the door frame square and undamaged, with only the closer, latch or screen worn?</t>
   </si>
   <si>
     <t xml:space="preserve">Door knob loose or falling off</t>
@@ -1883,7 +1882,7 @@
     <t xml:space="preserve">Are there outlets near the halls or stairs where you want lights?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There are outlets near the halls or stairs where you want lights</t>
+    <t xml:space="preserve">1. Are there outlets near the halls or stairs where you want lights?</t>
   </si>
   <si>
     <t xml:space="preserve">Assemble a bed frame</t>
@@ -1901,7 +1900,7 @@
     <t xml:space="preserve">Is it a standard bed frame, not a bunk, loft or storage bed?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is a standard bed frame, not a bunk, loft or storage bed</t>
+    <t xml:space="preserve">1. Is it a standard bed frame, not a bunk, loft or storage bed?</t>
   </si>
   <si>
     <t xml:space="preserve">Hook up a washer or electric dryer</t>
@@ -1922,7 +1921,7 @@
     <t xml:space="preserve">Are the water valves, drain standpipe and dryer outlet already in place?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The water valves, drain standpipe and dryer outlet are already in place</t>
+    <t xml:space="preserve">1. Are the water valves, drain standpipe and dryer outlet already in place?</t>
   </si>
   <si>
     <t xml:space="preserve">Mount a towel bar or toilet paper holder</t>
@@ -1943,7 +1942,7 @@
     <t xml:space="preserve">Is it towel or paper hardware, not a grab bar you will lean on?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is towel or paper hardware, not a grab bar you will lean on</t>
+    <t xml:space="preserve">1. Is it towel or paper hardware, not a grab bar you will lean on?</t>
   </si>
   <si>
     <t xml:space="preserve">Holes in exterior siding</t>
@@ -1967,8 +1966,7 @@
     <t xml:space="preserve">Are the holes smaller than a quarter, with solid siding around them?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The holes are smaller than a quarter
-- The siding around the holes is solid</t>
+    <t xml:space="preserve">1. Are the holes smaller than a quarter, with solid siding around them?</t>
   </si>
   <si>
     <t xml:space="preserve">Install a window AC unit</t>
@@ -1995,8 +1993,8 @@
     <t xml:space="preserve">Will an adult helper be home to help lift the unit into the window?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is a standard plug-in 120V unit, not a 240V or through-wall model
-- An adult helper will be home to help lift the unit into the window</t>
+    <t xml:space="preserve">1. Is it a standard plug-in 120V unit, not a 240V or through-wall model?
+2. Will an adult helper be home to help lift the unit into the window?</t>
   </si>
   <si>
     <t xml:space="preserve">Wobbly handrail or loose stair step</t>
@@ -2023,9 +2021,8 @@
     <t xml:space="preserve">Is this an indoor stair or low ground-level railing, not an elevated deck rail?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The railing or step is loose, but not cracked or rotted
-- It is not pulling out of the wall
-- It is an indoor stair or low ground-level railing, not an elevated deck rail</t>
+    <t xml:space="preserve">1. Is the railing or step loose but not cracked, rotted or pulling out of the wall?
+2. Is this an indoor stair or low ground-level railing, not an elevated deck rail?</t>
   </si>
   <si>
     <t xml:space="preserve">Loose or damaged baseboard or trim</t>
@@ -2046,7 +2043,7 @@
     <t xml:space="preserve">Is the damage limited to one or two short sections, not a whole room?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The damage is limited to one or two short sections, not a whole room</t>
+    <t xml:space="preserve">1. Is the damage limited to one or two short sections, not a whole room?</t>
   </si>
   <si>
     <t xml:space="preserve">Rotted trim by an exterior door or window</t>
@@ -2070,8 +2067,7 @@
     <t xml:space="preserve">Is the rot limited to about 4 feet of trim, with solid wood behind it?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The rot is limited to about 4 feet of trim
-- The wood behind the rotted trim is solid</t>
+    <t xml:space="preserve">1. Is the rot limited to about 4 feet of trim, with solid wood behind it?</t>
   </si>
   <si>
     <t xml:space="preserve">Cracked or missing grout</t>
@@ -2095,8 +2091,7 @@
     <t xml:space="preserve">Is the tile itself solid, with no loose tiles or soft spots in the wall?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The tile itself is solid, with no loose tiles
-- There are no soft spots in the wall</t>
+    <t xml:space="preserve">1. Is the tile itself solid, with no loose tiles or soft spots in the wall?</t>
   </si>
   <si>
     <t xml:space="preserve">Dripping shower or tub faucet</t>
@@ -2120,8 +2115,7 @@
     <t xml:space="preserve">Is the water dripping from the spout or handle, not from the wall or ceiling?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The water is dripping from the spout or handle
-- No water is coming from the wall or ceiling</t>
+    <t xml:space="preserve">1. Is the water dripping from the spout or handle, not from the wall or ceiling?</t>
   </si>
   <si>
     <t xml:space="preserve">Sliding patio door sticks or off track</t>
@@ -2145,8 +2139,7 @@
     <t xml:space="preserve">Are the door frame and track straight, with no bent metal or cracked glass?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The door frame and track are straight, with no bent metal
-- There is no cracked glass</t>
+    <t xml:space="preserve">1. Are the door frame and track straight, with no bent metal or cracked glass?</t>
   </si>
   <si>
     <t xml:space="preserve">Toilet rocks or leaks at the base</t>
@@ -2174,9 +2167,9 @@
 Will an adult helper be home to help lift the toilet?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The floor around the toilet is firm, not soft or spongy
-- Any leaking is from the base, not from the tank or supply line
-- An adult helper will be home to help lift the toilet</t>
+    <t xml:space="preserve">1. Is the floor around the toilet firm, not soft or spongy?
+2. Is the water coming from the base, not from the tank or supply line?
+3. Will an adult helper be home to help lift the toilet?</t>
   </si>
   <si>
     <t xml:space="preserve">Protect pipes and faucets from freezing</t>
@@ -2206,9 +2199,8 @@
     <t xml:space="preserve">Are all the pipes in a garage or open area, not an attic or crawlspace?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The pipes and faucets are thawed
-- There are no leaks right now
-- All the pipes are in a garage or open area, not an attic or crawlspace</t>
+    <t xml:space="preserve">1. Are the pipes and faucets thawed, with no leaks right now?
+2. Are all the pipes in a garage or open area, not an attic or crawlspace?</t>
   </si>
   <si>
     <t xml:space="preserve">Install a baby or pet gate</t>
@@ -2229,7 +2221,7 @@
     <t xml:space="preserve">Is the gate a hardware-mounted type that screws into the wall or post?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The gate is a hardware-mounted type that screws into the wall or post</t>
+    <t xml:space="preserve">1. Is the gate a hardware-mounted type that screws into the wall or post?</t>
   </si>
   <si>
     <t xml:space="preserve">Cracks in a walkway, patio or driveway</t>
@@ -2256,8 +2248,8 @@
     <t xml:space="preserve">Is the concrete level, with no sunken or raised slabs?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The cracks are about 1/2 inch wide or narrower
-- The concrete is level, with no sunken or raised slabs</t>
+    <t xml:space="preserve">1. Are the cracks about 1/2 inch wide or narrower?
+2. Is the concrete level, with no sunken or raised slabs?</t>
   </si>
   <si>
     <t xml:space="preserve">Secure tall furniture or a TV from tipping</t>
@@ -2278,7 +2270,7 @@
     <t xml:space="preserve">Is the wall drywall, not brick, stone or concrete?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The wall is drywall, not brick, stone or concrete</t>
+    <t xml:space="preserve">1. Is the wall drywall, not brick, stone or concrete?</t>
   </si>
   <si>
     <t xml:space="preserve">Assemble a dresser, wardrobe or bookcase</t>
@@ -2296,7 +2288,7 @@
     <t xml:space="preserve">Is it just one piece, not a large multi-door wardrobe?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is just one piece, not a large multi-door wardrobe</t>
+    <t xml:space="preserve">1. Is it just one piece, not a large multi-door wardrobe?</t>
   </si>
   <si>
     <t xml:space="preserve">Assemble a grill, patio set or gym gear</t>
@@ -2320,7 +2312,7 @@
     <t xml:space="preserve">Is it a single item, not a large machine that needs two people to build?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is a single item, not a large machine that needs two people to build</t>
+    <t xml:space="preserve">1. Is it a single item, not a large machine that needs two people to build?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a chandelier or hanging light</t>
@@ -2347,8 +2339,8 @@
     <t xml:space="preserve">Is there already a fixture hanging from the ceiling box in that spot?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The new fixture weighs about 35 pounds or less
-- There is already a fixture hanging from the ceiling box in that spot</t>
+    <t xml:space="preserve">1. Is the new fixture about 35 pounds or lighter?
+2. Is there already a fixture hanging from the ceiling box in that spot?</t>
   </si>
   <si>
     <t xml:space="preserve">Squeaky floor</t>
@@ -2372,7 +2364,7 @@
     <t xml:space="preserve">Are there only a few squeaky spots, not the whole floor?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There are only a few squeaky spots, not the whole floor</t>
+    <t xml:space="preserve">1. Are there only a few squeaky spots, not the whole floor?</t>
   </si>
   <si>
     <t xml:space="preserve">Stove burner or oven not heating</t>
@@ -2396,7 +2388,7 @@
     <t xml:space="preserve">Is it a coil burner or an oven element, not a flat glass cooktop?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is a coil burner or an oven element, not a flat glass cooktop</t>
+    <t xml:space="preserve">1. Is it a coil burner or an oven element, not a flat glass cooktop?</t>
   </si>
   <si>
     <t xml:space="preserve">Doorbell or chime not working</t>
@@ -2420,7 +2412,7 @@
     <t xml:space="preserve">Is there already a wired doorbell button and chime in place?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There is already a wired doorbell button and chime in place</t>
+    <t xml:space="preserve">1. Is there already a wired doorbell button and chime in place?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace the vent fan over the stove</t>
@@ -2447,8 +2439,8 @@
     <t xml:space="preserve">Will an adult helper be home to help hold the hood up?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The new hood is the same size and duct type as the old one
-- An adult helper will be home to help hold the hood up</t>
+    <t xml:space="preserve">1. Is the new hood the same size and duct type as the old one?
+2. Will an adult helper be home to help hold the hood up?</t>
   </si>
   <si>
     <t xml:space="preserve">Replace a porch or outdoor wall light</t>
@@ -2475,8 +2467,8 @@
     <t xml:space="preserve">Is there already a light fixture mounted at that spot?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The wiring in the box is dry and free of corrosion
-- There is already a light fixture mounted at that spot</t>
+    <t xml:space="preserve">1. Is the wiring in the box dry and free of corrosion?
+2. Is there already a light fixture mounted at that spot?</t>
   </si>
   <si>
     <t xml:space="preserve">Take apart and rebuild furniture for a move</t>
@@ -2497,8 +2489,7 @@
     <t xml:space="preserve">Is it 3 or fewer pieces, with no hauling or moving needed?</t>
   </si>
   <si>
-    <t xml:space="preserve">- There are 3 or fewer pieces
-- No hauling or moving is needed</t>
+    <t xml:space="preserve">1. Is it 3 or fewer pieces, with no hauling or moving needed?</t>
   </si>
   <si>
     <t xml:space="preserve">Blinds stuck, broken or won't go up</t>
@@ -2519,7 +2510,7 @@
     <t xml:space="preserve">Are the blinds standard store-bought blinds, not custom or motorized ones?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The blinds are standard store-bought, not custom or motorized</t>
+    <t xml:space="preserve">1. Are the blinds standard store-bought blinds, not custom or motorized ones?</t>
   </si>
   <si>
     <t xml:space="preserve">Door lock sticks or key won't turn</t>
@@ -2546,8 +2537,7 @@
     <t xml:space="preserve">Is the key intact, and can you still get in and out of the door?</t>
   </si>
   <si>
-    <t xml:space="preserve">- The key is intact
-- You can still get in and out of the door</t>
+    <t xml:space="preserve">1. Is the key intact, and can you still get in and out of the door?</t>
   </si>
   <si>
     <t xml:space="preserve">Appliance stopped working</t>
@@ -2574,7 +2564,7 @@
     <t xml:space="preserve">Is it a refrigerator, washer, dryer, dishwasher, oven or microwave?</t>
   </si>
   <si>
-    <t xml:space="preserve">- It is a refrigerator, washer, dryer, dishwasher, oven or microwave</t>
+    <t xml:space="preserve">1. Is it a refrigerator, washer, dryer, dishwasher, oven or microwave?</t>
   </si>
   <si>
     <t xml:space="preserve">Row count check</t>
@@ -6933,7 +6923,7 @@
     <t xml:space="preserve">Knockout questions</t>
   </si>
   <si>
-    <t xml:space="preserve">The conditions in the last column are PLACEHOLDER copy for design. In the one-job-at-a-time (wizard) version each task shows its conditions as a short list, then the same three overall conditions for every job (standard step ladder; only a swap or repair with no gas, new wiring or moved water lines; you have the part or fixture), then ONE question, "Does all of this apply to your job?" (Yes means it fits Fast Fix). There is no separate quick-check step in the wizard. Column Q is the single question the other versions ask instead; the next column keeps the questions that were merged or dropped on the way. A No flags that one task. Before booking, the member sees a page that separates the jobs that fit Fast Fix from the jobs that need a service request; everything goes in as one request, the fitting jobs are booked, and our team schedules the rest. When every job fits but the visit runs past 3 hours (up to 6), it is booked as two Fast Fix visits. Answers are not stored; they only route the request.</t>
+    <t xml:space="preserve">The questions in the last column are PLACEHOLDER copy for design. In the one-job-at-a-time (wizard) version each task asks its own questions (1 to 3), each answered on its own with Yes or No, followed by the same three overall questions for every job (standard step ladder; only a swap or repair with no gas, new wiring or moved water lines; you have the part or fixture), some with a Not sure option. There is no separate quick-check step in the wizard. Column Q is the single question the other versions ask instead; the next column keeps the questions that were merged or dropped on the way. A No or Not sure on any question marks that task as not eligible for Fast Fix. The member sees the jobs in two titled groups, Eligible for Fast Fix and Requires Service Request, schedules the eligible ones, and then submits the others as a service request from the confirmation page. When every job is eligible but the visit runs past 3 hours (up to 6), it is booked as two Fast Fix visits. Answers are not stored; they only route the request.</t>
   </si>
   <si>
     <t xml:space="preserve">Evidence limits (read this)</t>

</xml_diff>